<commit_message>
Clarify sensitivity assignment and finalize verified student workbook
</commit_message>
<xml_diff>
--- a/teaching/student-workbook.xlsx
+++ b/teaching/student-workbook.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision" sheetId="1" r:id="R783011fb6b064278"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="2" r:id="Re0cd86cc327f4b04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rent roll" sheetId="3" r:id="R06abe9fcb6cf4bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision" sheetId="1" r:id="R48e8585a09ab4506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="2" r:id="R3aa20ac16c374f25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rent roll" sheetId="3" r:id="R573cc9c8f0b54722"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -723,7 +723,7 @@
       <x:c r="D23" s="2"/>
       <x:c r="E23" s="2"/>
       <x:c r="F23" s="2" t="str">
-        <x:v>No debt, taxes, or credit losses.</x:v>
+        <x:v>No debt or income taxes. Credit losses excluded.</x:v>
       </x:c>
       <x:c r="G23" s="2"/>
       <x:c r="H23" s="2"/>

</xml_diff>